<commit_message>
get function and call stack working, organize files
</commit_message>
<xml_diff>
--- a/ISA attempt rriscv.xlsx
+++ b/ISA attempt rriscv.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmueller/Desktop/Seth/rrisc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0D061A8-ECC6-0449-8471-D95936B66CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F0C644-82A5-3F40-A592-45FB324A5DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="620" yWindow="760" windowWidth="29620" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="620" yWindow="760" windowWidth="29620" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="instructions" sheetId="1" r:id="rId1"/>
     <sheet name="registers" sheetId="2" r:id="rId2"/>
+    <sheet name="memory layout" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="162">
   <si>
     <t>maybe add later</t>
   </si>
@@ -401,6 +402,9 @@
     <t>constant 1</t>
   </si>
   <si>
+    <t>stack</t>
+  </si>
+  <si>
     <t>address of first unused memory</t>
   </si>
   <si>
@@ -416,26 +420,101 @@
     <t>stack pointer</t>
   </si>
   <si>
-    <t>locals pointer</t>
-  </si>
-  <si>
     <t>ARG</t>
   </si>
   <si>
-    <t>arguments pointer</t>
-  </si>
-  <si>
     <t>THIS</t>
   </si>
   <si>
     <t>THAT</t>
+  </si>
+  <si>
+    <t>result</t>
+  </si>
+  <si>
+    <t>push/pop segment</t>
+  </si>
+  <si>
+    <t>0-3</t>
+  </si>
+  <si>
+    <t>4-15</t>
+  </si>
+  <si>
+    <t>temp</t>
+  </si>
+  <si>
+    <t>static</t>
+  </si>
+  <si>
+    <t>16-255</t>
+  </si>
+  <si>
+    <t>256+</t>
+  </si>
+  <si>
+    <t>stack frame layout</t>
+  </si>
+  <si>
+    <t>return adress</t>
+  </si>
+  <si>
+    <t>Lcall_{self.current_file}_{name}</t>
+  </si>
+  <si>
+    <t>arg1</t>
+  </si>
+  <si>
+    <t>arg2</t>
+  </si>
+  <si>
+    <t>&lt;--- result written here</t>
+  </si>
+  <si>
+    <t>&lt;---- SP returned here</t>
+  </si>
+  <si>
+    <t>… previous stack …</t>
+  </si>
+  <si>
+    <t>prev LCL</t>
+  </si>
+  <si>
+    <t>prev ARG</t>
+  </si>
+  <si>
+    <t>prev THIS</t>
+  </si>
+  <si>
+    <t>prev THAT</t>
+  </si>
+  <si>
+    <t>local1</t>
+  </si>
+  <si>
+    <t>local2</t>
+  </si>
+  <si>
+    <t>local3</t>
+  </si>
+  <si>
+    <t>… current stack …</t>
+  </si>
+  <si>
+    <t>&lt;---- SP starts here</t>
+  </si>
+  <si>
+    <t>&lt;---- written back to arg1 on return</t>
+  </si>
+  <si>
+    <t>compiler reserved</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -464,8 +543,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -532,6 +619,12 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -554,7 +647,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -574,6 +667,19 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10162,16 +10268,25 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
+      <c r="B3" s="18" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1">
         <v>3</v>
       </c>
+      <c r="B4" s="18" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="1">
         <v>4</v>
       </c>
+      <c r="B5" s="18" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1">
@@ -10284,7 +10399,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10292,7 +10407,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10302,33 +10417,29 @@
       <c r="B29" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C29" s="18" t="s">
-        <v>133</v>
-      </c>
+      <c r="C29" s="18"/>
     </row>
     <row r="30" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="1">
         <v>29</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="C30" s="18" t="s">
-        <v>131</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="C30" s="18"/>
     </row>
     <row r="31" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="1">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10336,8 +10447,264 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FB6465B-E72D-0144-8CE3-5E7B7965A616}">
+  <dimension ref="A1:C51"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A1" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A2" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A3" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A4" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A5" s="20"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A6" s="20"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A7" s="20"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A8" s="20"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A9" s="20"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A10" s="20"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A11" s="20"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A12" s="20"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A13" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A14" s="20"/>
+      <c r="B14" s="18" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A15" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A16" s="20"/>
+      <c r="B16" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A17" s="20"/>
+      <c r="B17" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="C17" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A18" s="20"/>
+      <c r="B18" s="22" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A19" s="20"/>
+      <c r="B19" s="22" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A20" s="20"/>
+      <c r="B20" s="22" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A21" s="20"/>
+      <c r="B21" s="22" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A22" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A23" s="20"/>
+      <c r="B23" s="18" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A24" s="20"/>
+      <c r="B24" s="18" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="B25" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A26" s="19" t="s">
         <v>129</v>
       </c>
+      <c r="B26" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A27" s="20"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A28" s="20"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A29" s="20"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A30" s="20"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A31" s="20"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A32" s="20"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A33" s="20"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A34" s="20"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A35" s="20"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A36" s="20"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A37" s="20"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A38" s="20"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A39" s="20"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A40" s="20"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A41" s="20"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A42" s="20"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A43" s="20"/>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A44" s="20"/>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A45" s="20"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A46" s="20"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A47" s="21"/>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A48" s="21"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A49" s="21"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A50" s="21"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A51" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add tokenizer+parse and rename files
</commit_message>
<xml_diff>
--- a/ISA attempt rriscv.xlsx
+++ b/ISA attempt rriscv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmueller/Desktop/Seth/rrisc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F0C644-82A5-3F40-A592-45FB324A5DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D74014F-AEE5-0A41-8AC6-E4F5E92EE6BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="620" yWindow="760" windowWidth="29620" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="165">
   <si>
     <t>maybe add later</t>
   </si>
@@ -405,9 +405,6 @@
     <t>stack</t>
   </si>
   <si>
-    <t>address of first unused memory</t>
-  </si>
-  <si>
     <t>LCL</t>
   </si>
   <si>
@@ -423,12 +420,6 @@
     <t>ARG</t>
   </si>
   <si>
-    <t>THIS</t>
-  </si>
-  <si>
-    <t>THAT</t>
-  </si>
-  <si>
     <t>result</t>
   </si>
   <si>
@@ -508,6 +499,24 @@
   </si>
   <si>
     <t>compiler reserved</t>
+  </si>
+  <si>
+    <t>PTR2</t>
+  </si>
+  <si>
+    <t>PTR1</t>
+  </si>
+  <si>
+    <t>set with pop pointer 0</t>
+  </si>
+  <si>
+    <t>set with pop pointer 1</t>
+  </si>
+  <si>
+    <t>gray is memory addresses, first 4 are memory segments which can be used with push/pop `segment` `offset (int)` in byte code</t>
+  </si>
+  <si>
+    <t>address of first unused memory, push puts something here from a segment, pop moves the value at mem[SP-1] onto that memory segment at that index</t>
   </si>
 </sst>
 </file>
@@ -647,7 +656,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -680,6 +689,7 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10269,7 +10279,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10277,7 +10287,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10285,7 +10295,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10393,29 +10403,38 @@
       <c r="A26" s="1">
         <v>25</v>
       </c>
+      <c r="C26" s="22" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="1">
         <v>26</v>
       </c>
-      <c r="B27" s="18" t="s">
-        <v>134</v>
+      <c r="B27" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="1">
         <v>27</v>
       </c>
-      <c r="B28" s="18" t="s">
-        <v>133</v>
+      <c r="B28" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="1">
         <v>28</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>132</v>
+      <c r="B29" s="24" t="s">
+        <v>131</v>
       </c>
       <c r="C29" s="18"/>
     </row>
@@ -10423,8 +10442,8 @@
       <c r="A30" s="1">
         <v>29</v>
       </c>
-      <c r="B30" s="18" t="s">
-        <v>128</v>
+      <c r="B30" s="22" t="s">
+        <v>127</v>
       </c>
       <c r="C30" s="18"/>
     </row>
@@ -10432,14 +10451,14 @@
       <c r="A31" s="1">
         <v>30</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>129</v>
+      <c r="B31" s="24" t="s">
+        <v>128</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>127</v>
+        <v>164</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10447,7 +10466,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -10465,40 +10484,40 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A1" s="19" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A2" s="19" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A3" s="19" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A4" s="19" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>126</v>
@@ -10530,105 +10549,105 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A13" s="23" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A14" s="20"/>
       <c r="B14" s="18" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A15" s="19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A16" s="20"/>
       <c r="B16" s="18" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A17" s="20"/>
       <c r="B17" s="22" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C17" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A18" s="20"/>
       <c r="B18" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A19" s="20"/>
       <c r="B19" s="22" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A20" s="20"/>
       <c r="B20" s="22" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A21" s="20"/>
       <c r="B21" s="22" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A22" s="19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A23" s="20"/>
       <c r="B23" s="18" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A24" s="20"/>
       <c r="B24" s="18" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.15">
       <c r="B25" s="18" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A26" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.15">

</xml_diff>